<commit_message>
Add kompetensi_keahlian relation to Dudi model and views
Introduces a foreign key 'kompetensi_id' to the Dudi table and establishes a relationship between Dudi and Kompetensi_keahlian models. Updates Dudi import logic to associate imported records with the correct Kompetensi_keahlian, and modifies the index view to display the related kompetensi keahlian. Migration file is renamed and updated, and the seeder is cleaned up for consistency.
</commit_message>
<xml_diff>
--- a/excel/dudi_pkl.xlsx
+++ b/excel/dudi_pkl.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikko\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\pkl\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6B0B58-E237-4FDB-A90B-B4328C95B3EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47194211-9911-45BF-863C-7A23E0AF5190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="262">
   <si>
     <t>No</t>
   </si>
@@ -801,13 +799,34 @@
   </si>
   <si>
     <t>nomor Kepegawaian</t>
+  </si>
+  <si>
+    <t>Kompetensi Keahlian</t>
+  </si>
+  <si>
+    <t>Teknik Komputer dan Jaringan</t>
+  </si>
+  <si>
+    <t>Teknik Kendaraan Ringan</t>
+  </si>
+  <si>
+    <t>Teknik Sepeda Motor</t>
+  </si>
+  <si>
+    <t>Layanan Penunjang Kefarmasian Klinis dan Komunitas (LPK3)</t>
+  </si>
+  <si>
+    <t>Teknik Pengelasan</t>
+  </si>
+  <si>
+    <t>Teknik Elektronika Industri</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -822,6 +841,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9ECBFF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -859,7 +889,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -869,6 +899,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1160,6 +1202,7 @@
     <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="56.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -1187,7 +1230,9 @@
       <c r="H1" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="2"/>
+      <c r="I1" s="5" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
@@ -1204,7 +1249,9 @@
       <c r="H2" s="2">
         <v>12</v>
       </c>
-      <c r="I2" s="2"/>
+      <c r="I2" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -1221,7 +1268,9 @@
       <c r="H3" s="2">
         <v>3</v>
       </c>
-      <c r="I3" s="2"/>
+      <c r="I3" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -1238,7 +1287,9 @@
       <c r="H4" s="2">
         <v>10</v>
       </c>
-      <c r="I4" s="2"/>
+      <c r="I4" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -1261,7 +1312,9 @@
       <c r="H5" s="2">
         <v>5</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -1284,7 +1337,9 @@
       <c r="H6" s="2">
         <v>2</v>
       </c>
-      <c r="I6" s="2"/>
+      <c r="I6" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -1301,7 +1356,9 @@
       <c r="H7" s="2">
         <v>3</v>
       </c>
-      <c r="I7" s="2"/>
+      <c r="I7" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -1318,7 +1375,9 @@
       <c r="H8" s="2">
         <v>0</v>
       </c>
-      <c r="I8" s="2"/>
+      <c r="I8" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -1337,7 +1396,9 @@
       <c r="H9" s="2">
         <v>10</v>
       </c>
-      <c r="I9" s="2"/>
+      <c r="I9" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -1354,7 +1415,9 @@
       <c r="H10" s="2">
         <v>2</v>
       </c>
-      <c r="I10" s="2"/>
+      <c r="I10" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -1371,7 +1434,9 @@
       <c r="H11" s="2">
         <v>10</v>
       </c>
-      <c r="I11" s="2"/>
+      <c r="I11" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -1390,7 +1455,9 @@
       <c r="H12" s="2">
         <v>25</v>
       </c>
-      <c r="I12" s="2"/>
+      <c r="I12" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -1413,7 +1480,9 @@
       <c r="H13" s="2">
         <v>2</v>
       </c>
-      <c r="I13" s="2"/>
+      <c r="I13" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
@@ -1430,7 +1499,9 @@
       <c r="H14" s="2">
         <v>0</v>
       </c>
-      <c r="I14" s="2"/>
+      <c r="I14" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
@@ -1447,7 +1518,9 @@
       <c r="H15" s="2">
         <v>10</v>
       </c>
-      <c r="I15" s="2"/>
+      <c r="I15" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -1464,7 +1537,9 @@
       <c r="H16" s="2">
         <v>4</v>
       </c>
-      <c r="I16" s="2"/>
+      <c r="I16" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
@@ -1487,7 +1562,9 @@
       <c r="H17" s="2">
         <v>4</v>
       </c>
-      <c r="I17" s="2"/>
+      <c r="I17" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
@@ -1504,7 +1581,9 @@
       <c r="H18" s="2">
         <v>10</v>
       </c>
-      <c r="I18" s="2"/>
+      <c r="I18" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
@@ -1525,7 +1604,9 @@
       <c r="H19" s="2">
         <v>2</v>
       </c>
-      <c r="I19" s="2"/>
+      <c r="I19" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -1542,7 +1623,9 @@
       <c r="H20" s="2">
         <v>10</v>
       </c>
-      <c r="I20" s="2"/>
+      <c r="I20" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
@@ -1559,7 +1642,9 @@
       <c r="H21" s="2">
         <v>10</v>
       </c>
-      <c r="I21" s="2"/>
+      <c r="I21" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
@@ -1576,7 +1661,9 @@
       <c r="H22" s="2">
         <v>10</v>
       </c>
-      <c r="I22" s="2"/>
+      <c r="I22" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
@@ -1599,7 +1686,9 @@
       <c r="H23" s="2">
         <v>3</v>
       </c>
-      <c r="I23" s="2"/>
+      <c r="I23" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -1616,7 +1705,9 @@
       <c r="H24" s="2">
         <v>10</v>
       </c>
-      <c r="I24" s="2"/>
+      <c r="I24" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
@@ -1633,7 +1724,9 @@
       <c r="H25" s="2">
         <v>10</v>
       </c>
-      <c r="I25" s="2"/>
+      <c r="I25" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
@@ -1650,7 +1743,9 @@
       <c r="H26" s="2">
         <v>10</v>
       </c>
-      <c r="I26" s="2"/>
+      <c r="I26" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
@@ -1669,7 +1764,9 @@
       <c r="H27" s="2">
         <v>21</v>
       </c>
-      <c r="I27" s="2"/>
+      <c r="I27" s="8" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
@@ -1686,7 +1783,9 @@
       <c r="H28" s="2">
         <v>10</v>
       </c>
-      <c r="I28" s="2"/>
+      <c r="I28" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
@@ -1703,7 +1802,9 @@
       <c r="H29" s="2">
         <v>10</v>
       </c>
-      <c r="I29" s="2"/>
+      <c r="I29" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
@@ -1720,7 +1821,9 @@
       <c r="H30" s="2">
         <v>10</v>
       </c>
-      <c r="I30" s="2"/>
+      <c r="I30" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
@@ -1737,7 +1840,9 @@
       <c r="H31" s="2">
         <v>10</v>
       </c>
-      <c r="I31" s="2"/>
+      <c r="I31" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
@@ -1754,7 +1859,9 @@
       <c r="H32" s="2">
         <v>10</v>
       </c>
-      <c r="I32" s="2"/>
+      <c r="I32" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
@@ -1771,7 +1878,9 @@
       <c r="H33" s="2">
         <v>10</v>
       </c>
-      <c r="I33" s="2"/>
+      <c r="I33" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
@@ -1788,7 +1897,9 @@
       <c r="H34" s="2">
         <v>10</v>
       </c>
-      <c r="I34" s="2"/>
+      <c r="I34" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
@@ -1805,7 +1916,9 @@
       <c r="H35" s="2">
         <v>10</v>
       </c>
-      <c r="I35" s="2"/>
+      <c r="I35" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
@@ -1822,7 +1935,9 @@
       <c r="H36" s="2">
         <v>10</v>
       </c>
-      <c r="I36" s="2"/>
+      <c r="I36" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
@@ -1839,7 +1954,9 @@
       <c r="H37" s="2">
         <v>10</v>
       </c>
-      <c r="I37" s="2"/>
+      <c r="I37" s="8" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
@@ -1856,7 +1973,9 @@
       <c r="H38" s="2">
         <v>1</v>
       </c>
-      <c r="I38" s="2"/>
+      <c r="I38" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
@@ -1873,7 +1992,9 @@
       <c r="H39" s="2">
         <v>10</v>
       </c>
-      <c r="I39" s="2"/>
+      <c r="I39" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
@@ -1890,7 +2011,9 @@
       <c r="H40" s="2">
         <v>10</v>
       </c>
-      <c r="I40" s="2"/>
+      <c r="I40" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
@@ -1907,7 +2030,9 @@
       <c r="H41" s="2">
         <v>10</v>
       </c>
-      <c r="I41" s="2"/>
+      <c r="I41" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="2">
@@ -1924,7 +2049,9 @@
       <c r="H42" s="2">
         <v>10</v>
       </c>
-      <c r="I42" s="2"/>
+      <c r="I42" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="2">
@@ -1941,7 +2068,9 @@
       <c r="H43" s="2">
         <v>10</v>
       </c>
-      <c r="I43" s="2"/>
+      <c r="I43" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="2">
@@ -1958,7 +2087,9 @@
       <c r="H44" s="2">
         <v>10</v>
       </c>
-      <c r="I44" s="2"/>
+      <c r="I44" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="2">
@@ -1975,7 +2106,9 @@
       <c r="H45" s="2">
         <v>10</v>
       </c>
-      <c r="I45" s="2"/>
+      <c r="I45" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="2">
@@ -1992,7 +2125,9 @@
       <c r="H46" s="2">
         <v>10</v>
       </c>
-      <c r="I46" s="2"/>
+      <c r="I46" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="2">
@@ -2009,7 +2144,9 @@
       <c r="H47" s="2">
         <v>10</v>
       </c>
-      <c r="I47" s="2"/>
+      <c r="I47" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="2">
@@ -2026,7 +2163,9 @@
       <c r="H48" s="2">
         <v>10</v>
       </c>
-      <c r="I48" s="2"/>
+      <c r="I48" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
@@ -2043,7 +2182,9 @@
       <c r="H49" s="2">
         <v>10</v>
       </c>
-      <c r="I49" s="2"/>
+      <c r="I49" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="2">
@@ -2060,7 +2201,9 @@
       <c r="H50" s="2">
         <v>10</v>
       </c>
-      <c r="I50" s="2"/>
+      <c r="I50" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="2">
@@ -2077,7 +2220,9 @@
       <c r="H51" s="2">
         <v>10</v>
       </c>
-      <c r="I51" s="2"/>
+      <c r="I51" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="2">
@@ -2094,7 +2239,9 @@
       <c r="H52" s="2">
         <v>10</v>
       </c>
-      <c r="I52" s="2"/>
+      <c r="I52" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="2">
@@ -2111,7 +2258,9 @@
       <c r="H53" s="2">
         <v>10</v>
       </c>
-      <c r="I53" s="2"/>
+      <c r="I53" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="2">
@@ -2128,7 +2277,9 @@
       <c r="H54" s="2">
         <v>10</v>
       </c>
-      <c r="I54" s="2"/>
+      <c r="I54" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="2">
@@ -2145,7 +2296,9 @@
       <c r="H55" s="2">
         <v>10</v>
       </c>
-      <c r="I55" s="2"/>
+      <c r="I55" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="2">
@@ -2162,7 +2315,9 @@
       <c r="H56" s="2">
         <v>10</v>
       </c>
-      <c r="I56" s="2"/>
+      <c r="I56" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="2">
@@ -2179,7 +2334,9 @@
       <c r="H57" s="2">
         <v>10</v>
       </c>
-      <c r="I57" s="2"/>
+      <c r="I57" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="2">
@@ -2196,7 +2353,9 @@
       <c r="H58" s="2">
         <v>10</v>
       </c>
-      <c r="I58" s="2"/>
+      <c r="I58" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="2">
@@ -2213,7 +2372,9 @@
       <c r="H59" s="2">
         <v>10</v>
       </c>
-      <c r="I59" s="2"/>
+      <c r="I59" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="2">
@@ -2230,7 +2391,9 @@
       <c r="H60" s="2">
         <v>10</v>
       </c>
-      <c r="I60" s="2"/>
+      <c r="I60" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="2">
@@ -2247,7 +2410,9 @@
       <c r="H61" s="2">
         <v>10</v>
       </c>
-      <c r="I61" s="2"/>
+      <c r="I61" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="2">
@@ -2264,7 +2429,9 @@
       <c r="H62" s="2">
         <v>10</v>
       </c>
-      <c r="I62" s="2"/>
+      <c r="I62" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="2">
@@ -2281,7 +2448,9 @@
       <c r="H63" s="2">
         <v>10</v>
       </c>
-      <c r="I63" s="2"/>
+      <c r="I63" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="2">
@@ -2298,7 +2467,9 @@
       <c r="H64" s="2">
         <v>10</v>
       </c>
-      <c r="I64" s="2"/>
+      <c r="I64" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="2">
@@ -2315,7 +2486,9 @@
       <c r="H65" s="2">
         <v>10</v>
       </c>
-      <c r="I65" s="2"/>
+      <c r="I65" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="2">
@@ -2332,7 +2505,9 @@
       <c r="H66" s="2">
         <v>10</v>
       </c>
-      <c r="I66" s="2"/>
+      <c r="I66" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="2">
@@ -2349,7 +2524,9 @@
       <c r="H67" s="2">
         <v>10</v>
       </c>
-      <c r="I67" s="2"/>
+      <c r="I67" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="2">
@@ -2366,7 +2543,9 @@
       <c r="H68" s="2">
         <v>10</v>
       </c>
-      <c r="I68" s="2"/>
+      <c r="I68" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="2">
@@ -2383,7 +2562,9 @@
       <c r="H69" s="2">
         <v>10</v>
       </c>
-      <c r="I69" s="2"/>
+      <c r="I69" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="2">
@@ -2400,7 +2581,9 @@
       <c r="H70" s="2">
         <v>10</v>
       </c>
-      <c r="I70" s="2"/>
+      <c r="I70" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="2">
@@ -2417,7 +2600,9 @@
       <c r="H71" s="2">
         <v>10</v>
       </c>
-      <c r="I71" s="2"/>
+      <c r="I71" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="2">
@@ -2434,7 +2619,9 @@
       <c r="H72" s="2">
         <v>10</v>
       </c>
-      <c r="I72" s="2"/>
+      <c r="I72" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="2">
@@ -2451,7 +2638,9 @@
       <c r="H73" s="2">
         <v>10</v>
       </c>
-      <c r="I73" s="2"/>
+      <c r="I73" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="2">
@@ -2468,7 +2657,9 @@
       <c r="H74" s="2">
         <v>10</v>
       </c>
-      <c r="I74" s="2"/>
+      <c r="I74" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="2">
@@ -2485,7 +2676,9 @@
       <c r="H75" s="2">
         <v>10</v>
       </c>
-      <c r="I75" s="2"/>
+      <c r="I75" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="2">
@@ -2502,7 +2695,9 @@
       <c r="H76" s="2">
         <v>10</v>
       </c>
-      <c r="I76" s="2"/>
+      <c r="I76" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="2">
@@ -2519,7 +2714,9 @@
       <c r="H77" s="2">
         <v>10</v>
       </c>
-      <c r="I77" s="2"/>
+      <c r="I77" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="2">
@@ -2536,7 +2733,9 @@
       <c r="H78" s="2">
         <v>10</v>
       </c>
-      <c r="I78" s="2"/>
+      <c r="I78" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="2">
@@ -2553,7 +2752,9 @@
       <c r="H79" s="2">
         <v>10</v>
       </c>
-      <c r="I79" s="2"/>
+      <c r="I79" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="2">
@@ -2570,7 +2771,9 @@
       <c r="H80" s="2">
         <v>10</v>
       </c>
-      <c r="I80" s="2"/>
+      <c r="I80" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="2">
@@ -2587,7 +2790,9 @@
       <c r="H81" s="2">
         <v>10</v>
       </c>
-      <c r="I81" s="2"/>
+      <c r="I81" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="2">
@@ -2604,7 +2809,9 @@
       <c r="H82" s="2">
         <v>15</v>
       </c>
-      <c r="I82" s="2"/>
+      <c r="I82" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="2">
@@ -2621,7 +2828,9 @@
       <c r="H83" s="2">
         <v>10</v>
       </c>
-      <c r="I83" s="2"/>
+      <c r="I83" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="2">
@@ -2638,7 +2847,9 @@
       <c r="H84" s="2">
         <v>10</v>
       </c>
-      <c r="I84" s="2"/>
+      <c r="I84" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="2">
@@ -2655,7 +2866,9 @@
       <c r="H85" s="2">
         <v>10</v>
       </c>
-      <c r="I85" s="2"/>
+      <c r="I85" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="2">
@@ -2672,7 +2885,9 @@
       <c r="H86" s="2">
         <v>10</v>
       </c>
-      <c r="I86" s="2"/>
+      <c r="I86" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="2">
@@ -2689,7 +2904,9 @@
       <c r="H87" s="2">
         <v>10</v>
       </c>
-      <c r="I87" s="2"/>
+      <c r="I87" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="2">
@@ -2706,7 +2923,9 @@
       <c r="H88" s="2">
         <v>10</v>
       </c>
-      <c r="I88" s="2"/>
+      <c r="I88" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="2">
@@ -2723,7 +2942,9 @@
       <c r="H89" s="2">
         <v>10</v>
       </c>
-      <c r="I89" s="2"/>
+      <c r="I89" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="2">
@@ -2740,7 +2961,9 @@
       <c r="H90" s="2">
         <v>10</v>
       </c>
-      <c r="I90" s="2"/>
+      <c r="I90" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="2">
@@ -2757,7 +2980,9 @@
       <c r="H91" s="2">
         <v>10</v>
       </c>
-      <c r="I91" s="2"/>
+      <c r="I91" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="2">
@@ -2774,7 +2999,9 @@
       <c r="H92" s="2">
         <v>10</v>
       </c>
-      <c r="I92" s="2"/>
+      <c r="I92" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="2">
@@ -2791,7 +3018,9 @@
       <c r="H93" s="2">
         <v>10</v>
       </c>
-      <c r="I93" s="2"/>
+      <c r="I93" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="2">
@@ -2808,7 +3037,9 @@
       <c r="H94" s="2">
         <v>10</v>
       </c>
-      <c r="I94" s="2"/>
+      <c r="I94" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="2">
@@ -2825,7 +3056,9 @@
       <c r="H95" s="2">
         <v>10</v>
       </c>
-      <c r="I95" s="2"/>
+      <c r="I95" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="2">
@@ -2842,7 +3075,9 @@
       <c r="H96" s="2">
         <v>10</v>
       </c>
-      <c r="I96" s="2"/>
+      <c r="I96" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="2">
@@ -2859,7 +3094,9 @@
       <c r="H97" s="2">
         <v>10</v>
       </c>
-      <c r="I97" s="2"/>
+      <c r="I97" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="2">
@@ -2876,7 +3113,9 @@
       <c r="H98" s="2">
         <v>10</v>
       </c>
-      <c r="I98" s="2"/>
+      <c r="I98" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="2">
@@ -2893,7 +3132,9 @@
       <c r="H99" s="2">
         <v>10</v>
       </c>
-      <c r="I99" s="2"/>
+      <c r="I99" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="2">
@@ -2910,7 +3151,9 @@
       <c r="H100" s="2">
         <v>10</v>
       </c>
-      <c r="I100" s="2"/>
+      <c r="I100" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="2">
@@ -2927,7 +3170,9 @@
       <c r="H101" s="2">
         <v>10</v>
       </c>
-      <c r="I101" s="2"/>
+      <c r="I101" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="2">
@@ -2944,7 +3189,9 @@
       <c r="H102" s="2">
         <v>10</v>
       </c>
-      <c r="I102" s="2"/>
+      <c r="I102" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="2">
@@ -2961,7 +3208,9 @@
       <c r="H103" s="2">
         <v>10</v>
       </c>
-      <c r="I103" s="2"/>
+      <c r="I103" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="2">
@@ -2978,7 +3227,9 @@
       <c r="H104" s="2">
         <v>10</v>
       </c>
-      <c r="I104" s="2"/>
+      <c r="I104" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="2">
@@ -2995,7 +3246,9 @@
       <c r="H105" s="2">
         <v>10</v>
       </c>
-      <c r="I105" s="2"/>
+      <c r="I105" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="2">
@@ -3012,7 +3265,9 @@
       <c r="H106" s="2">
         <v>10</v>
       </c>
-      <c r="I106" s="2"/>
+      <c r="I106" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="2">
@@ -3029,7 +3284,9 @@
       <c r="H107" s="2">
         <v>10</v>
       </c>
-      <c r="I107" s="2"/>
+      <c r="I107" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="2">
@@ -3046,7 +3303,9 @@
       <c r="H108" s="2">
         <v>10</v>
       </c>
-      <c r="I108" s="2"/>
+      <c r="I108" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="2">
@@ -3063,7 +3322,9 @@
       <c r="H109" s="2">
         <v>10</v>
       </c>
-      <c r="I109" s="2"/>
+      <c r="I109" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="2">
@@ -3080,7 +3341,9 @@
       <c r="H110" s="2">
         <v>10</v>
       </c>
-      <c r="I110" s="2"/>
+      <c r="I110" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="2">
@@ -3097,7 +3360,9 @@
       <c r="H111" s="2">
         <v>10</v>
       </c>
-      <c r="I111" s="2"/>
+      <c r="I111" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="2">
@@ -3114,7 +3379,9 @@
       <c r="H112" s="2">
         <v>10</v>
       </c>
-      <c r="I112" s="2"/>
+      <c r="I112" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="2">
@@ -3131,7 +3398,9 @@
       <c r="H113" s="2">
         <v>10</v>
       </c>
-      <c r="I113" s="2"/>
+      <c r="I113" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="2">
@@ -3148,7 +3417,9 @@
       <c r="H114" s="2">
         <v>10</v>
       </c>
-      <c r="I114" s="2"/>
+      <c r="I114" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="2">
@@ -3165,7 +3436,9 @@
       <c r="H115" s="2">
         <v>10</v>
       </c>
-      <c r="I115" s="2"/>
+      <c r="I115" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="2">
@@ -3182,7 +3455,9 @@
       <c r="H116" s="2">
         <v>10</v>
       </c>
-      <c r="I116" s="2"/>
+      <c r="I116" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="2">
@@ -3199,7 +3474,9 @@
       <c r="H117" s="2">
         <v>10</v>
       </c>
-      <c r="I117" s="2"/>
+      <c r="I117" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="2">
@@ -3216,7 +3493,9 @@
       <c r="H118" s="2">
         <v>10</v>
       </c>
-      <c r="I118" s="2"/>
+      <c r="I118" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="2">
@@ -3233,7 +3512,9 @@
       <c r="H119" s="2">
         <v>10</v>
       </c>
-      <c r="I119" s="2"/>
+      <c r="I119" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="2">
@@ -3250,7 +3531,9 @@
       <c r="H120" s="2">
         <v>10</v>
       </c>
-      <c r="I120" s="2"/>
+      <c r="I120" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="2">
@@ -3267,7 +3550,9 @@
       <c r="H121" s="2">
         <v>10</v>
       </c>
-      <c r="I121" s="2"/>
+      <c r="I121" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="2">
@@ -3284,7 +3569,9 @@
       <c r="H122" s="2">
         <v>10</v>
       </c>
-      <c r="I122" s="2"/>
+      <c r="I122" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="2">
@@ -3301,7 +3588,9 @@
       <c r="H123" s="2">
         <v>10</v>
       </c>
-      <c r="I123" s="2"/>
+      <c r="I123" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="2">
@@ -3318,7 +3607,9 @@
       <c r="H124" s="2">
         <v>10</v>
       </c>
-      <c r="I124" s="2"/>
+      <c r="I124" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="2">
@@ -3335,7 +3626,9 @@
       <c r="H125" s="2">
         <v>10</v>
       </c>
-      <c r="I125" s="2"/>
+      <c r="I125" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="2">
@@ -3354,7 +3647,9 @@
       <c r="H126" s="2">
         <v>10</v>
       </c>
-      <c r="I126" s="2"/>
+      <c r="I126" s="8" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="2">
@@ -3373,7 +3668,9 @@
       <c r="H127" s="2">
         <v>10</v>
       </c>
-      <c r="I127" s="2"/>
+      <c r="I127" s="8" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="2">
@@ -3392,7 +3689,9 @@
       <c r="H128" s="2">
         <v>10</v>
       </c>
-      <c r="I128" s="2"/>
+      <c r="I128" s="8" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="2">
@@ -3411,7 +3710,9 @@
       <c r="H129" s="2">
         <v>10</v>
       </c>
-      <c r="I129" s="2"/>
+      <c r="I129" s="8" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="2">
@@ -3428,7 +3729,9 @@
       <c r="H130" s="2">
         <v>10</v>
       </c>
-      <c r="I130" s="2"/>
+      <c r="I130" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="2">
@@ -3445,7 +3748,9 @@
       <c r="H131" s="2">
         <v>10</v>
       </c>
-      <c r="I131" s="2"/>
+      <c r="I131" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
@@ -3462,7 +3767,9 @@
       <c r="H132" s="2">
         <v>10</v>
       </c>
-      <c r="I132" s="2"/>
+      <c r="I132" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="2">
@@ -3479,7 +3786,9 @@
       <c r="H133" s="2">
         <v>10</v>
       </c>
-      <c r="I133" s="2"/>
+      <c r="I133" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="2">
@@ -3496,7 +3805,9 @@
       <c r="H134" s="2">
         <v>10</v>
       </c>
-      <c r="I134" s="2"/>
+      <c r="I134" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="2">
@@ -3513,7 +3824,9 @@
       <c r="H135" s="2">
         <v>10</v>
       </c>
-      <c r="I135" s="2"/>
+      <c r="I135" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="2">
@@ -3530,7 +3843,9 @@
       <c r="H136" s="2">
         <v>10</v>
       </c>
-      <c r="I136" s="2"/>
+      <c r="I136" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="2">
@@ -3547,7 +3862,9 @@
       <c r="H137" s="2">
         <v>10</v>
       </c>
-      <c r="I137" s="2"/>
+      <c r="I137" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="2">
@@ -3564,7 +3881,9 @@
       <c r="H138" s="2">
         <v>10</v>
       </c>
-      <c r="I138" s="2"/>
+      <c r="I138" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="2">
@@ -3581,7 +3900,9 @@
       <c r="H139" s="2">
         <v>10</v>
       </c>
-      <c r="I139" s="2"/>
+      <c r="I139" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="2">
@@ -3600,7 +3921,9 @@
       <c r="H140" s="2">
         <v>10</v>
       </c>
-      <c r="I140" s="2"/>
+      <c r="I140" s="7" t="s">
+        <v>260</v>
+      </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="2">
@@ -3619,7 +3942,9 @@
       <c r="H141" s="2">
         <v>10</v>
       </c>
-      <c r="I141" s="2"/>
+      <c r="I141" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="2">
@@ -3638,7 +3963,9 @@
       <c r="H142" s="2">
         <v>10</v>
       </c>
-      <c r="I142" s="2"/>
+      <c r="I142" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="2">
@@ -3655,7 +3982,9 @@
       <c r="H143" s="2">
         <v>30</v>
       </c>
-      <c r="I143" s="2"/>
+      <c r="I143" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="2">
@@ -3674,7 +4003,9 @@
       <c r="H144" s="2">
         <v>10</v>
       </c>
-      <c r="I144" s="2"/>
+      <c r="I144" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="2">
@@ -3693,7 +4024,9 @@
       <c r="H145" s="2">
         <v>5</v>
       </c>
-      <c r="I145" s="2"/>
+      <c r="I145" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="2">
@@ -3712,7 +4045,9 @@
       <c r="H146" s="2">
         <v>3</v>
       </c>
-      <c r="I146" s="2"/>
+      <c r="I146" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="2">
@@ -3733,7 +4068,9 @@
       <c r="H147" s="2">
         <v>3</v>
       </c>
-      <c r="I147" s="2"/>
+      <c r="I147" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="2">
@@ -3754,7 +4091,9 @@
       <c r="H148" s="2">
         <v>1</v>
       </c>
-      <c r="I148" s="2"/>
+      <c r="I148" s="8" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="2">
@@ -3777,7 +4116,9 @@
       <c r="H149" s="2">
         <v>3</v>
       </c>
-      <c r="I149" s="2"/>
+      <c r="I149" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="2">
@@ -3800,7 +4141,9 @@
       <c r="H150" s="2">
         <v>2</v>
       </c>
-      <c r="I150" s="2"/>
+      <c r="I150" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="2">
@@ -3819,7 +4162,9 @@
       <c r="H151" s="2">
         <v>3</v>
       </c>
-      <c r="I151" s="2"/>
+      <c r="I151" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="2">
@@ -3834,7 +4179,9 @@
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
-      <c r="I152" s="2"/>
+      <c r="I152" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" s="2">
@@ -3853,7 +4200,9 @@
       <c r="H153" s="2">
         <v>5</v>
       </c>
-      <c r="I153" s="2"/>
+      <c r="I153" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="2">
@@ -3872,7 +4221,9 @@
       <c r="H154" s="2">
         <v>10</v>
       </c>
-      <c r="I154" s="2"/>
+      <c r="I154" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="2">
@@ -3891,7 +4242,9 @@
       <c r="H155" s="2">
         <v>10</v>
       </c>
-      <c r="I155" s="2"/>
+      <c r="I155" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="2">
@@ -3910,7 +4263,9 @@
       <c r="H156" s="2">
         <v>10</v>
       </c>
-      <c r="I156" s="2"/>
+      <c r="I156" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="2">
@@ -3929,7 +4284,9 @@
       <c r="H157" s="2">
         <v>10</v>
       </c>
-      <c r="I157" s="2"/>
+      <c r="I157" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" s="2">
@@ -3946,7 +4303,9 @@
       <c r="H158" s="2">
         <v>10</v>
       </c>
-      <c r="I158" s="2"/>
+      <c r="I158" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" s="2">
@@ -3965,7 +4324,9 @@
       <c r="H159" s="2">
         <v>3</v>
       </c>
-      <c r="I159" s="2"/>
+      <c r="I159" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" s="2">
@@ -3984,7 +4345,9 @@
       <c r="H160" s="2">
         <v>5</v>
       </c>
-      <c r="I160" s="2"/>
+      <c r="I160" s="8" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="2">
@@ -4003,7 +4366,9 @@
       <c r="H161" s="2">
         <v>2</v>
       </c>
-      <c r="I161" s="2"/>
+      <c r="I161" s="8" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="2">
@@ -4022,8 +4387,8 @@
       <c r="F162" s="2"/>
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
-      <c r="I162" s="2">
-        <v>5</v>
+      <c r="I162" s="6" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
@@ -4043,7 +4408,9 @@
       <c r="H163" s="2">
         <v>5</v>
       </c>
-      <c r="I163" s="2"/>
+      <c r="I163" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="2">
@@ -4062,7 +4429,9 @@
       <c r="H164" s="2">
         <v>5</v>
       </c>
-      <c r="I164" s="2"/>
+      <c r="I164" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="2">
@@ -4081,7 +4450,9 @@
       <c r="H165" s="2">
         <v>2</v>
       </c>
-      <c r="I165" s="2"/>
+      <c r="I165" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="2">
@@ -4100,7 +4471,9 @@
       <c r="H166" s="2">
         <v>2</v>
       </c>
-      <c r="I166" s="2"/>
+      <c r="I166" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="2">
@@ -4119,7 +4492,9 @@
       <c r="H167" s="2">
         <v>5</v>
       </c>
-      <c r="I167" s="2"/>
+      <c r="I167" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="2">
@@ -4138,7 +4513,9 @@
       <c r="H168" s="2">
         <v>3</v>
       </c>
-      <c r="I168" s="2"/>
+      <c r="I168" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="2">
@@ -4155,7 +4532,9 @@
       <c r="H169" s="2">
         <v>3</v>
       </c>
-      <c r="I169" s="2"/>
+      <c r="I169" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" s="2">
@@ -4172,7 +4551,9 @@
       <c r="H170" s="2">
         <v>2</v>
       </c>
-      <c r="I170" s="2"/>
+      <c r="I170" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" s="2">
@@ -4191,7 +4572,9 @@
       <c r="H171" s="2">
         <v>5</v>
       </c>
-      <c r="I171" s="2"/>
+      <c r="I171" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="2">
@@ -4210,7 +4593,9 @@
       <c r="H172" s="2">
         <v>3</v>
       </c>
-      <c r="I172" s="2"/>
+      <c r="I172" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" s="2">
@@ -4229,7 +4614,9 @@
       <c r="H173" s="2">
         <v>5</v>
       </c>
-      <c r="I173" s="2"/>
+      <c r="I173" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="2">
@@ -4248,7 +4635,9 @@
       <c r="H174" s="2">
         <v>3</v>
       </c>
-      <c r="I174" s="2"/>
+      <c r="I174" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" s="2">
@@ -4267,7 +4656,9 @@
       <c r="H175" s="2">
         <v>5</v>
       </c>
-      <c r="I175" s="2"/>
+      <c r="I175" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" s="2">
@@ -4286,7 +4677,9 @@
       <c r="H176" s="2">
         <v>3</v>
       </c>
-      <c r="I176" s="2"/>
+      <c r="I176" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" s="2">
@@ -4303,7 +4696,9 @@
       <c r="H177" s="2">
         <v>3</v>
       </c>
-      <c r="I177" s="2"/>
+      <c r="I177" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" s="2">
@@ -4320,7 +4715,9 @@
       <c r="H178" s="2">
         <v>3</v>
       </c>
-      <c r="I178" s="2"/>
+      <c r="I178" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" s="2">
@@ -4337,7 +4734,9 @@
       <c r="H179" s="2">
         <v>3</v>
       </c>
-      <c r="I179" s="2"/>
+      <c r="I179" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" s="2">
@@ -4354,7 +4753,9 @@
       <c r="H180" s="2">
         <v>2</v>
       </c>
-      <c r="I180" s="2"/>
+      <c r="I180" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="2">
@@ -4373,7 +4774,9 @@
       <c r="H181" s="2">
         <v>2</v>
       </c>
-      <c r="I181" s="2"/>
+      <c r="I181" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="2">
@@ -4392,7 +4795,9 @@
       <c r="H182" s="2">
         <v>3</v>
       </c>
-      <c r="I182" s="2"/>
+      <c r="I182" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" s="2">
@@ -4409,7 +4814,9 @@
       <c r="H183" s="2">
         <v>4</v>
       </c>
-      <c r="I183" s="2"/>
+      <c r="I183" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" s="2">
@@ -4426,7 +4833,9 @@
       <c r="H184" s="2">
         <v>2</v>
       </c>
-      <c r="I184" s="2"/>
+      <c r="I184" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" s="2">
@@ -4445,7 +4854,9 @@
       <c r="H185" s="2">
         <v>5</v>
       </c>
-      <c r="I185" s="2"/>
+      <c r="I185" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" s="2">
@@ -4462,7 +4873,9 @@
       <c r="H186" s="2">
         <v>3</v>
       </c>
-      <c r="I186" s="2"/>
+      <c r="I186" s="6" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" s="2">
@@ -4483,7 +4896,9 @@
       <c r="H187" s="2">
         <v>1</v>
       </c>
-      <c r="I187" s="2"/>
+      <c r="I187" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" s="2">
@@ -4500,7 +4915,9 @@
       <c r="H188" s="2">
         <v>2</v>
       </c>
-      <c r="I188" s="2"/>
+      <c r="I188" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" s="2">
@@ -4517,7 +4934,9 @@
       <c r="H189" s="2">
         <v>2</v>
       </c>
-      <c r="I189" s="2"/>
+      <c r="I189" s="7" t="s">
+        <v>261</v>
+      </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" s="2">
@@ -4534,7 +4953,9 @@
       <c r="H190" s="2">
         <v>2</v>
       </c>
-      <c r="I190" s="2"/>
+      <c r="I190" s="8" t="s">
+        <v>256</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>